<commit_message>
refactor: update data processing logic, improve UI filtering, and add Docker environment configuration
</commit_message>
<xml_diff>
--- a/top_20_maiores_variacoes_formatado.xlsx
+++ b/top_20_maiores_variacoes_formatado.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ricar\OneDrive\Área de Trabalho\visdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ricar\OneDrive\Área de Trabalho\Python\mirante\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB18F0EE-27A6-46CD-83F2-8E1C2CEC8A07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFE446AD-B914-4AB0-873E-3F7290977BDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-30" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Top 20 - PCD" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="84">
   <si>
     <t>Codigo</t>
   </si>
@@ -56,21 +56,9 @@
     <t>Mai/2025</t>
   </si>
   <si>
-    <t>113.036</t>
-  </si>
-  <si>
-    <t>3.059</t>
-  </si>
-  <si>
     <t>Mar/2025</t>
   </si>
   <si>
-    <t>109.977</t>
-  </si>
-  <si>
-    <t>1.985</t>
-  </si>
-  <si>
     <t>RIO DE JANEIRO</t>
   </si>
   <si>
@@ -80,160 +68,52 @@
     <t>Jun/2025</t>
   </si>
   <si>
-    <t>78.672</t>
-  </si>
-  <si>
-    <t>1.965</t>
-  </si>
-  <si>
     <t>Jul/2024</t>
   </si>
   <si>
     <t>Ago/2024</t>
   </si>
   <si>
-    <t>106.907</t>
-  </si>
-  <si>
-    <t>1.749</t>
-  </si>
-  <si>
     <t>Mai/2024</t>
   </si>
   <si>
     <t>Jun/2024</t>
   </si>
   <si>
-    <t>103.801</t>
-  </si>
-  <si>
-    <t>1.711</t>
-  </si>
-  <si>
-    <t>76.707</t>
-  </si>
-  <si>
-    <t>1.610</t>
-  </si>
-  <si>
     <t>Nov/2024</t>
   </si>
   <si>
     <t>Dez/2024</t>
   </si>
   <si>
-    <t>110.468</t>
-  </si>
-  <si>
-    <t>1.608</t>
-  </si>
-  <si>
     <t>FORTALEZA</t>
   </si>
   <si>
     <t>CE</t>
   </si>
   <si>
-    <t>70.868</t>
-  </si>
-  <si>
-    <t>1.604</t>
-  </si>
-  <si>
     <t>Abr/2024</t>
   </si>
   <si>
-    <t>102.090</t>
-  </si>
-  <si>
-    <t>1.553</t>
-  </si>
-  <si>
-    <t>114.574</t>
-  </si>
-  <si>
-    <t>1.538</t>
-  </si>
-  <si>
-    <t>69.264</t>
-  </si>
-  <si>
-    <t>1.476</t>
-  </si>
-  <si>
-    <t>75.097</t>
-  </si>
-  <si>
-    <t>1.462</t>
-  </si>
-  <si>
-    <t>66.972</t>
-  </si>
-  <si>
-    <t>1.455</t>
-  </si>
-  <si>
-    <t>59.771</t>
-  </si>
-  <si>
-    <t>1.452</t>
-  </si>
-  <si>
     <t>Out/2025</t>
   </si>
   <si>
     <t>Nov/2025</t>
   </si>
   <si>
-    <t>114.357</t>
-  </si>
-  <si>
-    <t>-1.442</t>
-  </si>
-  <si>
     <t>RECIFE</t>
   </si>
   <si>
     <t>PE</t>
   </si>
   <si>
-    <t>51.729</t>
-  </si>
-  <si>
-    <t>1.425</t>
-  </si>
-  <si>
-    <t>68.393</t>
-  </si>
-  <si>
-    <t>1.421</t>
-  </si>
-  <si>
     <t>Fev/2025</t>
   </si>
   <si>
-    <t>107.992</t>
-  </si>
-  <si>
-    <t>-1.382</t>
-  </si>
-  <si>
-    <t>105.158</t>
-  </si>
-  <si>
-    <t>1.357</t>
-  </si>
-  <si>
     <t>SALVADOR</t>
   </si>
   <si>
     <t>BA</t>
-  </si>
-  <si>
-    <t>54.283</t>
-  </si>
-  <si>
-    <t>1.352</t>
   </si>
   <si>
     <t>Idosos Atual</t>
@@ -448,11 +328,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -756,17 +637,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23.21875" customWidth="1"/>
-    <col min="3" max="3" width="22.77734375" customWidth="1"/>
-    <col min="4" max="4" width="16.6640625" customWidth="1"/>
-    <col min="5" max="5" width="15.6640625" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="25.33203125" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="4" max="4" width="15.140625" customWidth="1"/>
+    <col min="6" max="6" width="17.28515625" customWidth="1"/>
+    <col min="7" max="7" width="25.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -789,7 +668,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>355030</v>
       </c>
@@ -805,114 +684,114 @@
       <c r="E2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="2">
+        <v>113036</v>
+      </c>
+      <c r="G2" s="2">
+        <v>3059</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>355030</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
         <v>11</v>
-      </c>
-      <c r="G2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>355030</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" t="s">
-        <v>13</v>
       </c>
       <c r="E3" t="s">
         <v>9</v>
       </c>
-      <c r="F3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F3" s="2">
+        <v>109977</v>
+      </c>
+      <c r="G3" s="2">
+        <v>1985</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>330455</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D4" t="s">
         <v>10</v>
       </c>
       <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="2">
+        <v>78672</v>
+      </c>
+      <c r="G4" s="2">
+        <v>1965</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>355030</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="2">
+        <v>106907</v>
+      </c>
+      <c r="G5" s="2">
+        <v>1749</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>355030</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" t="s">
         <v>18</v>
       </c>
-      <c r="F4" t="s">
-        <v>19</v>
-      </c>
-      <c r="G4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>355030</v>
-      </c>
-      <c r="B5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" t="s">
-        <v>22</v>
-      </c>
-      <c r="F5" t="s">
-        <v>23</v>
-      </c>
-      <c r="G5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>355030</v>
-      </c>
-      <c r="B6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D6" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" t="s">
-        <v>26</v>
-      </c>
-      <c r="F6" t="s">
-        <v>27</v>
-      </c>
-      <c r="G6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F6" s="2">
+        <v>103801</v>
+      </c>
+      <c r="G6" s="2">
+        <v>1711</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>330455</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D7" t="s">
         <v>9</v>
@@ -920,14 +799,14 @@
       <c r="E7" t="s">
         <v>10</v>
       </c>
-      <c r="F7" t="s">
-        <v>29</v>
-      </c>
-      <c r="G7" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F7" s="2">
+        <v>76707</v>
+      </c>
+      <c r="G7" s="2">
+        <v>1610</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>355030</v>
       </c>
@@ -938,42 +817,42 @@
         <v>8</v>
       </c>
       <c r="D8" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E8" t="s">
-        <v>32</v>
-      </c>
-      <c r="F8" t="s">
-        <v>33</v>
-      </c>
-      <c r="G8" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+      <c r="F8" s="2">
+        <v>110468</v>
+      </c>
+      <c r="G8" s="2">
+        <v>1608</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>230440</v>
       </c>
       <c r="B9" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="C9" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="D9" t="s">
         <v>10</v>
       </c>
       <c r="E9" t="s">
-        <v>18</v>
-      </c>
-      <c r="F9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+      <c r="F9" s="2">
+        <v>70868</v>
+      </c>
+      <c r="G9" s="2">
+        <v>1604</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>355030</v>
       </c>
@@ -984,19 +863,19 @@
         <v>8</v>
       </c>
       <c r="D10" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="E10" t="s">
-        <v>25</v>
-      </c>
-      <c r="F10" t="s">
-        <v>40</v>
-      </c>
-      <c r="G10" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+      <c r="F10" s="2">
+        <v>102090</v>
+      </c>
+      <c r="G10" s="2">
+        <v>1553</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>355030</v>
       </c>
@@ -1010,24 +889,24 @@
         <v>10</v>
       </c>
       <c r="E11" t="s">
-        <v>18</v>
-      </c>
-      <c r="F11" t="s">
-        <v>42</v>
-      </c>
-      <c r="G11" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+      <c r="F11" s="2">
+        <v>114574</v>
+      </c>
+      <c r="G11" s="2">
+        <v>1538</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>230440</v>
       </c>
       <c r="B12" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="C12" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="D12" t="s">
         <v>9</v>
@@ -1035,114 +914,114 @@
       <c r="E12" t="s">
         <v>10</v>
       </c>
-      <c r="F12" t="s">
-        <v>44</v>
-      </c>
-      <c r="G12" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F12" s="2">
+        <v>69264</v>
+      </c>
+      <c r="G12" s="2">
+        <v>1476</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>330455</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D13" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E13" t="s">
         <v>9</v>
       </c>
-      <c r="F13" t="s">
-        <v>46</v>
-      </c>
-      <c r="G13" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F13" s="2">
+        <v>75097</v>
+      </c>
+      <c r="G13" s="2">
+        <v>1462</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>330455</v>
       </c>
       <c r="B14" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" t="s">
         <v>17</v>
       </c>
-      <c r="D14" t="s">
-        <v>25</v>
-      </c>
       <c r="E14" t="s">
-        <v>26</v>
-      </c>
-      <c r="F14" t="s">
-        <v>48</v>
-      </c>
-      <c r="G14" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+      <c r="F14" s="2">
+        <v>66972</v>
+      </c>
+      <c r="G14" s="2">
+        <v>1455</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>230440</v>
       </c>
       <c r="B15" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="C15" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="D15" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="E15" t="s">
+        <v>17</v>
+      </c>
+      <c r="F15" s="2">
+        <v>59771</v>
+      </c>
+      <c r="G15" s="2">
+        <v>1452</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>355030</v>
+      </c>
+      <c r="B16" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" t="s">
+        <v>24</v>
+      </c>
+      <c r="E16" t="s">
         <v>25</v>
       </c>
-      <c r="F15" t="s">
-        <v>50</v>
-      </c>
-      <c r="G15" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16">
-        <v>355030</v>
-      </c>
-      <c r="B16" t="s">
-        <v>7</v>
-      </c>
-      <c r="C16" t="s">
-        <v>8</v>
-      </c>
-      <c r="D16" t="s">
-        <v>52</v>
-      </c>
-      <c r="E16" t="s">
-        <v>53</v>
-      </c>
-      <c r="F16" t="s">
-        <v>54</v>
-      </c>
-      <c r="G16" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F16" s="2">
+        <v>114357</v>
+      </c>
+      <c r="G16" s="2">
+        <v>-1442</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>261160</v>
       </c>
       <c r="B17" t="s">
-        <v>56</v>
+        <v>26</v>
       </c>
       <c r="C17" t="s">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="D17" t="s">
         <v>9</v>
@@ -1150,37 +1029,37 @@
       <c r="E17" t="s">
         <v>10</v>
       </c>
-      <c r="F17" t="s">
-        <v>58</v>
-      </c>
-      <c r="G17" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F17" s="2">
+        <v>51729</v>
+      </c>
+      <c r="G17" s="2">
+        <v>1425</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>330455</v>
       </c>
       <c r="B18" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C18" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D18" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E18" t="s">
-        <v>21</v>
-      </c>
-      <c r="F18" t="s">
-        <v>60</v>
-      </c>
-      <c r="G18" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+      <c r="F18" s="2">
+        <v>68393</v>
+      </c>
+      <c r="G18" s="2">
+        <v>1421</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>355030</v>
       </c>
@@ -1191,19 +1070,19 @@
         <v>8</v>
       </c>
       <c r="D19" t="s">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="E19" t="s">
-        <v>13</v>
-      </c>
-      <c r="F19" t="s">
-        <v>63</v>
-      </c>
-      <c r="G19" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="F19" s="2">
+        <v>107992</v>
+      </c>
+      <c r="G19" s="2">
+        <v>-1382</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>355030</v>
       </c>
@@ -1214,27 +1093,27 @@
         <v>8</v>
       </c>
       <c r="D20" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E20" t="s">
-        <v>21</v>
-      </c>
-      <c r="F20" t="s">
-        <v>65</v>
-      </c>
-      <c r="G20" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+      <c r="F20" s="2">
+        <v>105158</v>
+      </c>
+      <c r="G20" s="2">
+        <v>1357</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>292740</v>
       </c>
       <c r="B21" t="s">
-        <v>67</v>
+        <v>29</v>
       </c>
       <c r="C21" t="s">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="D21" t="s">
         <v>9</v>
@@ -1242,11 +1121,11 @@
       <c r="E21" t="s">
         <v>10</v>
       </c>
-      <c r="F21" t="s">
-        <v>69</v>
-      </c>
-      <c r="G21" t="s">
-        <v>70</v>
+      <c r="F21" s="2">
+        <v>54283</v>
+      </c>
+      <c r="G21" s="2">
+        <v>1352</v>
       </c>
     </row>
   </sheetData>
@@ -1257,16 +1136,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="17" customWidth="1"/>
-    <col min="4" max="4" width="20.109375" customWidth="1"/>
-    <col min="5" max="5" width="17.33203125" customWidth="1"/>
-    <col min="6" max="6" width="16.5546875" customWidth="1"/>
-    <col min="7" max="7" width="18.33203125" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1283,13 +1155,13 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>71</v>
+        <v>31</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>355030</v>
       </c>
@@ -1300,19 +1172,19 @@
         <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>73</v>
+        <v>33</v>
       </c>
       <c r="E2" t="s">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="F2" t="s">
-        <v>74</v>
+        <v>34</v>
       </c>
       <c r="G2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>355030</v>
       </c>
@@ -1323,19 +1195,19 @@
         <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>76</v>
+        <v>36</v>
       </c>
       <c r="E3" t="s">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="F3" t="s">
-        <v>77</v>
+        <v>37</v>
       </c>
       <c r="G3" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>355030</v>
       </c>
@@ -1346,19 +1218,19 @@
         <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="E4" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="F4" t="s">
-        <v>79</v>
+        <v>39</v>
       </c>
       <c r="G4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>355030</v>
       </c>
@@ -1369,19 +1241,19 @@
         <v>8</v>
       </c>
       <c r="D5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E5" t="s">
         <v>9</v>
       </c>
       <c r="F5" t="s">
-        <v>81</v>
+        <v>41</v>
       </c>
       <c r="G5" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>355030</v>
       </c>
@@ -1395,39 +1267,39 @@
         <v>10</v>
       </c>
       <c r="E6" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F6" t="s">
-        <v>83</v>
+        <v>43</v>
       </c>
       <c r="G6" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>330455</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D7" t="s">
-        <v>73</v>
+        <v>33</v>
       </c>
       <c r="E7" t="s">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="F7" t="s">
-        <v>85</v>
+        <v>45</v>
       </c>
       <c r="G7" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>355030</v>
       </c>
@@ -1444,44 +1316,44 @@
         <v>10</v>
       </c>
       <c r="F8" t="s">
-        <v>87</v>
+        <v>47</v>
       </c>
       <c r="G8" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>330455</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D9" t="s">
         <v>10</v>
       </c>
       <c r="E9" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F9" t="s">
-        <v>89</v>
+        <v>49</v>
       </c>
       <c r="G9" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>330455</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C10" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D10" t="s">
         <v>9</v>
@@ -1490,13 +1362,13 @@
         <v>10</v>
       </c>
       <c r="F10" t="s">
-        <v>91</v>
+        <v>51</v>
       </c>
       <c r="G10" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>355030</v>
       </c>
@@ -1507,111 +1379,111 @@
         <v>8</v>
       </c>
       <c r="D11" t="s">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="E11" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F11" t="s">
-        <v>93</v>
+        <v>53</v>
       </c>
       <c r="G11" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>330455</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D12" t="s">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="E12" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="F12" t="s">
-        <v>95</v>
+        <v>55</v>
       </c>
       <c r="G12" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>330455</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D13" t="s">
-        <v>76</v>
+        <v>36</v>
       </c>
       <c r="E13" t="s">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="F13" t="s">
-        <v>97</v>
+        <v>57</v>
       </c>
       <c r="G13" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>330455</v>
       </c>
       <c r="B14" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D14" t="s">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="E14" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F14" t="s">
-        <v>99</v>
+        <v>59</v>
       </c>
       <c r="G14" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>330455</v>
       </c>
       <c r="B15" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C15" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D15" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E15" t="s">
         <v>9</v>
       </c>
       <c r="F15" t="s">
-        <v>101</v>
+        <v>61</v>
       </c>
       <c r="G15" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>355030</v>
       </c>
@@ -1622,65 +1494,65 @@
         <v>8</v>
       </c>
       <c r="D16" t="s">
-        <v>103</v>
+        <v>63</v>
       </c>
       <c r="E16" t="s">
-        <v>104</v>
+        <v>64</v>
       </c>
       <c r="F16" t="s">
-        <v>105</v>
+        <v>65</v>
       </c>
       <c r="G16" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>500270</v>
       </c>
       <c r="B17" t="s">
-        <v>107</v>
+        <v>67</v>
       </c>
       <c r="C17" t="s">
-        <v>108</v>
+        <v>68</v>
       </c>
       <c r="D17" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E17" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F17" t="s">
-        <v>109</v>
+        <v>69</v>
       </c>
       <c r="G17" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>211130</v>
       </c>
       <c r="B18" t="s">
-        <v>111</v>
+        <v>71</v>
       </c>
       <c r="C18" t="s">
-        <v>112</v>
+        <v>72</v>
       </c>
       <c r="D18" t="s">
+        <v>33</v>
+      </c>
+      <c r="E18" t="s">
+        <v>28</v>
+      </c>
+      <c r="F18" t="s">
         <v>73</v>
       </c>
-      <c r="E18" t="s">
-        <v>62</v>
-      </c>
-      <c r="F18" t="s">
-        <v>113</v>
-      </c>
       <c r="G18" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>355030</v>
       </c>
@@ -1691,19 +1563,19 @@
         <v>8</v>
       </c>
       <c r="D19" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="E19" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F19" t="s">
-        <v>115</v>
+        <v>75</v>
       </c>
       <c r="G19" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>355030</v>
       </c>
@@ -1714,39 +1586,39 @@
         <v>8</v>
       </c>
       <c r="D20" t="s">
-        <v>104</v>
+        <v>64</v>
       </c>
       <c r="E20" t="s">
-        <v>117</v>
+        <v>77</v>
       </c>
       <c r="F20" t="s">
-        <v>118</v>
+        <v>78</v>
       </c>
       <c r="G20" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>510180</v>
       </c>
       <c r="B21" t="s">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="C21" t="s">
-        <v>121</v>
+        <v>81</v>
       </c>
       <c r="D21" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E21" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F21" t="s">
-        <v>122</v>
+        <v>82</v>
       </c>
       <c r="G21" t="s">
-        <v>123</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>